<commit_message>
feat: attach catalog plans during studio data import
Resolve monthly/quarterly plan names on batches and plan names on enrollments and invoices so imports can create BatchPlans, memberships, and purchaseMeta links.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/apps/step-up/public/templates/studio-import-template.xlsx
+++ b/apps/step-up/public/templates/studio-import-template.xlsx
@@ -227,6 +227,16 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Monthly plan name</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Quarterly plan name</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -293,6 +303,16 @@
       <c r="N2" t="inlineStr">
         <is>
           <t>Active</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Kids Monthly</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Kids Quarterly</t>
         </is>
       </c>
     </row>
@@ -448,6 +468,11 @@
           <t>End reason</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Plan name</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -472,6 +497,11 @@
       </c>
       <c r="E2"/>
       <c r="F2"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Kids Monthly</t>
+        </is>
+      </c>
     </row>
   </sheetData>
 </worksheet>
@@ -531,6 +561,11 @@
           <t>Refunded at</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Plan name</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -579,6 +614,11 @@
         </is>
       </c>
       <c r="J2"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Kids Monthly</t>
+        </is>
+      </c>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>

<commit_message>
feat: enhance date handling in student and studio import processes
- Updated date parsing to support dd/mm/yyyy format in both student and studio import modules, ensuring compatibility with Excel date formats.
- Introduced functions to maintain local calendar days during date processing, preventing unintended shifts when converting to ISO format.
- Enhanced tests to validate new date handling logic, ensuring accurate parsing and formatting of enrollment and session dates.
- Updated import templates and documentation to reflect the new date format requirements.
</commit_message>
<xml_diff>
--- a/apps/step-up/public/templates/studio-import-template.xlsx
+++ b/apps/step-up/public/templates/studio-import-template.xlsx
@@ -1,20 +1,421 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <sheets>
-    <sheet name="Students" sheetId="1" r:id="rId1"/>
-    <sheet name="Locations" sheetId="2" r:id="rId2"/>
-    <sheet name="Batches" sheetId="3" r:id="rId3"/>
-    <sheet name="Sessions" sheetId="4" r:id="rId4"/>
-    <sheet name="Enrollments" sheetId="5" r:id="rId5"/>
-    <sheet name="Invoices &amp; Payments" sheetId="6" r:id="rId6"/>
-    <sheet name="Attendance" sheetId="7" r:id="rId7"/>
+    <sheet name="Students" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Locations" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Batches" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Sessions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Enrollments" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Invoices &amp; Payments" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Attendance" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
+  <definedNames/>
 </workbook>
+</file>
+
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
+</styleSheet>
+</file>
+
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -64,14 +465,20 @@
           <t>28</t>
         </is>
       </c>
-      <c r="E2"/>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -146,15 +553,20 @@
           <t>Parking</t>
         </is>
       </c>
-      <c r="G2"/>
-      <c r="H2"/>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -281,15 +693,14 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2024-06-03</t>
+          <t>03/06/2024</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2025-03-31</t>
-        </is>
-      </c>
-      <c r="K2"/>
+          <t>31/03/2025</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr">
         <is>
           <t>12</t>
@@ -317,11 +728,18 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -368,7 +786,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2024-06-03</t>
+          <t>03/06/2024</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -405,7 +823,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2024-06-05</t>
+          <t>05/06/2024</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -428,14 +846,20 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="G3"/>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -487,7 +911,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2024-06-01</t>
+          <t>01/06/2024</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -495,8 +919,6 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="E2"/>
-      <c r="F2"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>Kids Monthly</t>
@@ -504,11 +926,18 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -595,7 +1024,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2024-06-01</t>
+          <t>01/06/2024</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -613,7 +1042,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="J2"/>
       <c r="K2" t="inlineStr">
         <is>
           <t>Kids Monthly</t>
@@ -621,11 +1049,18 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -667,7 +1102,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2024-06-03</t>
+          <t>03/06/2024</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -682,5 +1117,6 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: enhance studio import functionality with day times support
- Added support for parsing and validating per-weekday day times in studio import templates, allowing for more flexible scheduling.
- Updated the data import service to handle day times in batch schedules, ensuring accurate data storage and retrieval.
- Introduced new DTOs and validation for day times, improving data integrity during imports.
- Enhanced unit tests to cover new day times functionality, ensuring robustness and reliability of the import process.
</commit_message>
<xml_diff>
--- a/apps/step-up/public/templates/studio-import-template.xlsx
+++ b/apps/step-up/public/templates/studio-import-template.xlsx
@@ -1,421 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Students" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Locations" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Batches" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Sessions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Enrollments" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Invoices &amp; Payments" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Attendance" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Students" sheetId="1" r:id="rId1"/>
+    <sheet name="Locations" sheetId="2" r:id="rId2"/>
+    <sheet name="Batches" sheetId="3" r:id="rId3"/>
+    <sheet name="Sessions" sheetId="4" r:id="rId4"/>
+    <sheet name="Enrollments" sheetId="5" r:id="rId5"/>
+    <sheet name="Invoices &amp; Payments" sheetId="6" r:id="rId6"/>
+    <sheet name="Attendance" sheetId="7" r:id="rId7"/>
   </sheets>
-  <definedNames/>
 </workbook>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-  </fonts>
-  <fills count="2">
-    <fill>
-      <patternFill/>
-    </fill>
-    <fill>
-      <patternFill patternType="gray125"/>
-    </fill>
-  </fills>
-  <borders count="1">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-  </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-  </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-  </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
-  </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
-</styleSheet>
-</file>
-
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="1F497D"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="EEECE1"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="4F81BD"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="C0504D"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="9BBB59"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="8064A2"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="4BACC6"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="F79646"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0000FF"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="800080"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme name="Office">
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="40000">
-              <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-</a:theme>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -465,20 +64,14 @@
           <t>28</t>
         </is>
       </c>
+      <c r="E2"/>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -553,20 +146,15 @@
           <t>Parking</t>
         </is>
       </c>
+      <c r="G2"/>
+      <c r="H2"/>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:P2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -611,40 +199,45 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>Day times</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>Start date</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>End date</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>UTC offset minutes</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Capacity</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Enrollment mode</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Monthly plan name</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Quarterly plan name</t>
         </is>
@@ -693,53 +286,52 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>03/06/2024</t>
+          <t>Mon 16:00-17:00, Wed 18:00-19:00</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>31/03/2025</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
+          <t>2024-06-03</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2025-03-31</t>
+        </is>
+      </c>
+      <c r="L2"/>
+      <c r="M2" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Staff only</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>Kids Monthly</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>Kids Quarterly</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -786,7 +378,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>03/06/2024</t>
+          <t>2024-06-03</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -823,7 +415,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>05/06/2024</t>
+          <t>2024-06-05</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -846,20 +438,14 @@
           <t>Regular</t>
         </is>
       </c>
+      <c r="G3"/>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -911,7 +497,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>01/06/2024</t>
+          <t>2024-06-01</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -919,6 +505,8 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="E2"/>
+      <c r="F2"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>Kids Monthly</t>
@@ -926,18 +514,11 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1024,7 +605,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>01/06/2024</t>
+          <t>2024-06-01</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1042,6 +623,7 @@
           <t>0</t>
         </is>
       </c>
+      <c r="J2"/>
       <c r="K2" t="inlineStr">
         <is>
           <t>Kids Monthly</t>
@@ -1049,18 +631,11 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1102,7 +677,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>03/06/2024</t>
+          <t>2024-06-03</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1117,6 +692,5 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>